<commit_message>
framework tourism world 2/8
</commit_message>
<xml_diff>
--- a/outputs/world/views_single_sheet.xlsx
+++ b/outputs/world/views_single_sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,33 +450,1083 @@
       <c r="H3" t="n">
         <v>2022</v>
       </c>
+      <c r="I3" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.05987</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.07005</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.55753</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.63815</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.24652</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.68666</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2.23272</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2.34605</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.99537</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3.9861</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.97426</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.85284</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.35015</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.16005</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.0574</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5.50139</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>5.49858</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>5.7128</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B8" t="n">
         <v>2.88621</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C8" t="n">
         <v>2.9547</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D8" t="n">
         <v>2.9604</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E8" t="n">
         <v>3.01889</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F8" t="n">
         <v>2.1474</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G8" t="n">
         <v>2.76457</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H8" t="n">
         <v>2.96775</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_arrivals_by_region_12_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2020.9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2272.5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2485.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2546.2</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="D17" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>439.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>491.4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>544.3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>586.5</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.236</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2.471</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2.955</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3.195</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>South Asia (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="F20" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2.083</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.056</v>
+      </c>
+      <c r="I20" t="n">
+        <v>9.523</v>
+      </c>
+      <c r="J20" t="n">
+        <v>14.355</v>
+      </c>
+      <c r="K20" t="n">
+        <v>16.029</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>262.6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>271.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>272.5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>284.2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>73.902</v>
+      </c>
+      <c r="H21" t="n">
+        <v>62.351</v>
+      </c>
+      <c r="I21" t="n">
+        <v>195.241</v>
+      </c>
+      <c r="J21" t="n">
+        <v>234.123</v>
+      </c>
+      <c r="K21" t="n">
+        <v>252.546</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3508.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3889.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4084.7</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4142</v>
+      </c>
+      <c r="G22" t="n">
+        <v>797.258</v>
+      </c>
+      <c r="H22" t="n">
+        <v>873.521</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3045.921</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3800.781</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4250.701</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3488.9</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3888.7</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3964.8</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3962.6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>579.165</v>
+      </c>
+      <c r="H23" t="n">
+        <v>313.499</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1202.564</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2329.21</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2700.05</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>26568.4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>27635.3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>28681.2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>29489.2</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10594.872</v>
+      </c>
+      <c r="H24" t="n">
+        <v>10047.669</v>
+      </c>
+      <c r="I24" t="n">
+        <v>23043.584</v>
+      </c>
+      <c r="J24" t="n">
+        <v>27129.43</v>
+      </c>
+      <c r="K24" t="n">
+        <v>28794.97</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>673.1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>660.8</v>
+      </c>
+      <c r="E25" t="n">
+        <v>636</v>
+      </c>
+      <c r="F25" t="n">
+        <v>604.3</v>
+      </c>
+      <c r="G25" t="n">
+        <v>95.996</v>
+      </c>
+      <c r="H25" t="n">
+        <v>165.966</v>
+      </c>
+      <c r="I25" t="n">
+        <v>404.707</v>
+      </c>
+      <c r="J25" t="n">
+        <v>483.885</v>
+      </c>
+      <c r="K25" t="n">
+        <v>489.689</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>South Asia (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>231.2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>268.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>289.7</v>
+      </c>
+      <c r="F26" t="n">
+        <v>307.1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>55.831</v>
+      </c>
+      <c r="H26" t="n">
+        <v>42.545</v>
+      </c>
+      <c r="I26" t="n">
+        <v>160.263</v>
+      </c>
+      <c r="J26" t="n">
+        <v>232.398</v>
+      </c>
+      <c r="K26" t="n">
+        <v>278.701</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1243</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1314.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1235.9</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1340</v>
+      </c>
+      <c r="G27" t="n">
+        <v>262.945</v>
+      </c>
+      <c r="H27" t="n">
+        <v>250.284</v>
+      </c>
+      <c r="I27" t="n">
+        <v>830.221</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1025.13128294283</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1297.90576947888</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4573.9</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5866</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6370.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>7092.1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1320.48</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1867.265</v>
+      </c>
+      <c r="I28" t="n">
+        <v>6359.413</v>
+      </c>
+      <c r="J28" t="n">
+        <v>8470.624000010759</v>
+      </c>
+      <c r="K28" t="n">
+        <v>9428.970904708071</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1904.7</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2299</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2560.7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2977</v>
+      </c>
+      <c r="G29" t="n">
+        <v>562.403</v>
+      </c>
+      <c r="H29" t="n">
+        <v>230.302</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1086.684</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2360.18863897558</v>
+      </c>
+      <c r="K29" t="n">
+        <v>2817.03795662791</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>67047.39999999999</v>
+      </c>
+      <c r="D30" t="n">
+        <v>71695.89999999999</v>
+      </c>
+      <c r="E30" t="n">
+        <v>71903.89999999999</v>
+      </c>
+      <c r="F30" t="n">
+        <v>71377.8</v>
+      </c>
+      <c r="G30" t="n">
+        <v>16676.276</v>
+      </c>
+      <c r="H30" t="n">
+        <v>28505.919</v>
+      </c>
+      <c r="I30" t="n">
+        <v>62765.346</v>
+      </c>
+      <c r="J30" t="n">
+        <v>72386.9099346476</v>
+      </c>
+      <c r="K30" t="n">
+        <v>79114.75530078731</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>386.7</v>
+      </c>
+      <c r="D31" t="n">
+        <v>466.4</v>
+      </c>
+      <c r="E31" t="n">
+        <v>416.3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>424.7</v>
+      </c>
+      <c r="G31" t="n">
+        <v>76.34399999999999</v>
+      </c>
+      <c r="H31" t="n">
+        <v>281.162</v>
+      </c>
+      <c r="I31" t="n">
+        <v>416.759</v>
+      </c>
+      <c r="J31" t="n">
+        <v>617.95432944935</v>
+      </c>
+      <c r="K31" t="n">
+        <v>765.914310277042</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>South Asia (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>159.3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>227</v>
+      </c>
+      <c r="E32" t="n">
+        <v>321</v>
+      </c>
+      <c r="F32" t="n">
+        <v>297.5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>34.655</v>
+      </c>
+      <c r="H32" t="n">
+        <v>45.87</v>
+      </c>
+      <c r="I32" t="n">
+        <v>200.859</v>
+      </c>
+      <c r="J32" t="n">
+        <v>308.24178665693</v>
+      </c>
+      <c r="K32" t="n">
+        <v>334.712612593961</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>574.301</v>
+      </c>
+      <c r="D33" t="n">
+        <v>585.447</v>
+      </c>
+      <c r="E33" t="n">
+        <v>597.803</v>
+      </c>
+      <c r="F33" t="n">
+        <v>566.6</v>
+      </c>
+      <c r="G33" t="n">
+        <v>107.201</v>
+      </c>
+      <c r="H33" t="n">
+        <v>153.671</v>
+      </c>
+      <c r="I33" t="n">
+        <v>366.029</v>
+      </c>
+      <c r="J33" t="n">
+        <v>529.515</v>
+      </c>
+      <c r="K33" t="n">
+        <v>586.16</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>46459.207</v>
+      </c>
+      <c r="D34" t="n">
+        <v>46675.98</v>
+      </c>
+      <c r="E34" t="n">
+        <v>48966.068</v>
+      </c>
+      <c r="F34" t="n">
+        <v>48061.7</v>
+      </c>
+      <c r="G34" t="n">
+        <v>13952.619</v>
+      </c>
+      <c r="H34" t="n">
+        <v>18293.477</v>
+      </c>
+      <c r="I34" t="n">
+        <v>33573.32</v>
+      </c>
+      <c r="J34" t="n">
+        <v>42840.828</v>
+      </c>
+      <c r="K34" t="n">
+        <v>46039.515</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>11764.684</v>
+      </c>
+      <c r="D35" t="n">
+        <v>12260.961</v>
+      </c>
+      <c r="E35" t="n">
+        <v>11952.945</v>
+      </c>
+      <c r="F35" t="n">
+        <v>12183.9</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2027.749</v>
+      </c>
+      <c r="H35" t="n">
+        <v>816.227</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3455.282</v>
+      </c>
+      <c r="J35" t="n">
+        <v>6726.311</v>
+      </c>
+      <c r="K35" t="n">
+        <v>7951.807</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>15505.744</v>
+      </c>
+      <c r="D36" t="n">
+        <v>15633.303</v>
+      </c>
+      <c r="E36" t="n">
+        <v>16082.513</v>
+      </c>
+      <c r="F36" t="n">
+        <v>16381.9</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2612.223</v>
+      </c>
+      <c r="H36" t="n">
+        <v>2259.032</v>
+      </c>
+      <c r="I36" t="n">
+        <v>11567.835</v>
+      </c>
+      <c r="J36" t="n">
+        <v>13771.831</v>
+      </c>
+      <c r="K36" t="n">
+        <v>14854.886</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>681.191</v>
+      </c>
+      <c r="D37" t="n">
+        <v>550.013</v>
+      </c>
+      <c r="E37" t="n">
+        <v>576.227</v>
+      </c>
+      <c r="F37" t="n">
+        <v>577.1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>127.276</v>
+      </c>
+      <c r="H37" t="n">
+        <v>227.801</v>
+      </c>
+      <c r="I37" t="n">
+        <v>366.673</v>
+      </c>
+      <c r="J37" t="n">
+        <v>463.179</v>
+      </c>
+      <c r="K37" t="n">
+        <v>459.545</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>South Asia (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1422.361</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1481.042</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1570.362</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1670.5</v>
+      </c>
+      <c r="G38" t="n">
+        <v>384.746</v>
+      </c>
+      <c r="H38" t="n">
+        <v>528.2569999999999</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1440.26</v>
+      </c>
+      <c r="J38" t="n">
+        <v>2016.472</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2496.501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
framework tourism world 4/8
</commit_message>
<xml_diff>
--- a/outputs/world/views_single_sheet.xlsx
+++ b/outputs/world/views_single_sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,301 +450,336 @@
       <c r="H3" t="n">
         <v>2022</v>
       </c>
-      <c r="I3" t="n">
-        <v>2023</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.05987</v>
+        <v>3.99537</v>
       </c>
       <c r="C4" t="n">
-        <v>2.07005</v>
+        <v>3.9861</v>
       </c>
       <c r="D4" t="n">
-        <v>2.55753</v>
+        <v>3.97426</v>
       </c>
       <c r="E4" t="n">
-        <v>2.63815</v>
+        <v>3.85284</v>
       </c>
       <c r="F4" t="n">
-        <v>1.24652</v>
+        <v>2.35015</v>
       </c>
       <c r="G4" t="n">
-        <v>1.68666</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2.23272</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2.34605</v>
-      </c>
+        <v>2.16005</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.99537</v>
+        <v>6.5</v>
       </c>
       <c r="C5" t="n">
-        <v>3.9861</v>
+        <v>6.6</v>
       </c>
       <c r="D5" t="n">
-        <v>3.97426</v>
+        <v>6.7</v>
       </c>
       <c r="E5" t="n">
-        <v>3.85284</v>
+        <v>6.8</v>
       </c>
       <c r="F5" t="n">
-        <v>2.35015</v>
+        <v>5.0574</v>
       </c>
       <c r="G5" t="n">
-        <v>2.16005</v>
+        <v>5.50139</v>
       </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>6.5</v>
-      </c>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>6.7</v>
-      </c>
+        <v>5.49858</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5.0574</v>
-      </c>
-      <c r="G6" t="n">
-        <v>5.50139</v>
-      </c>
+        <v>5.7128</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.88621</v>
+      </c>
       <c r="C7" t="n">
-        <v>5.49858</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>2.9547</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.9604</v>
+      </c>
       <c r="E7" t="n">
-        <v>5.7128</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2.88621</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2.9547</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2.9604</v>
-      </c>
-      <c r="E8" t="n">
         <v>3.01889</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F7" t="n">
         <v>2.1474</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G7" t="n">
         <v>2.76457</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H7" t="n">
         <v>2.96775</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>UN_Tourism_inbound_arrivals_by_region_12_2025</t>
-        </is>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_arrivals_by_purpose_12_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2024</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>geo</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>series</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2016</v>
+        <v>5703.7</v>
       </c>
       <c r="D14" t="n">
-        <v>2017</v>
+        <v>5706.7</v>
       </c>
       <c r="E14" t="n">
-        <v>2018</v>
+        <v>5636.8</v>
       </c>
       <c r="F14" t="n">
-        <v>2019</v>
+        <v>6112.7</v>
       </c>
       <c r="G14" t="n">
-        <v>2020</v>
+        <v>1565.465</v>
       </c>
       <c r="H14" t="n">
-        <v>2021</v>
+        <v>2270.304</v>
       </c>
       <c r="I14" t="n">
-        <v>2022</v>
+        <v>4952.511</v>
       </c>
       <c r="J14" t="n">
-        <v>2023</v>
+        <v>4973.06749958168</v>
       </c>
       <c r="K14" t="n">
-        <v>2024</v>
+        <v>5253.19541783694</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Africa (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.8</v>
+        <v>69611.3</v>
       </c>
       <c r="D15" t="n">
-        <v>3.7</v>
+        <v>76161.7</v>
       </c>
       <c r="E15" t="n">
-        <v>3.5</v>
+        <v>77171.60000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+        <v>77396.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>17367.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>28910.5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>66706.8</v>
+      </c>
+      <c r="J15" t="n">
+        <v>80195.98247311771</v>
+      </c>
+      <c r="K15" t="n">
+        <v>88506.1014367087</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Americas (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2020.9</v>
+        <v>14649</v>
       </c>
       <c r="D16" t="n">
-        <v>2272.5</v>
+        <v>14537</v>
       </c>
       <c r="E16" t="n">
-        <v>2485.8</v>
+        <v>14377.6</v>
       </c>
       <c r="F16" t="n">
-        <v>2546.2</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+        <v>14875.2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6766</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8326</v>
+      </c>
+      <c r="I16" t="n">
+        <v>10259</v>
+      </c>
+      <c r="J16" t="n">
+        <v>11321</v>
+      </c>
+      <c r="K16" t="n">
+        <v>11247</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>54.4</v>
+        <v>70275</v>
       </c>
       <c r="D17" t="n">
-        <v>58.4</v>
+        <v>75394</v>
       </c>
       <c r="E17" t="n">
-        <v>61.4</v>
+        <v>78850.89999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+        <v>80523.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>18423</v>
+      </c>
+      <c r="H17" t="n">
+        <v>18562</v>
+      </c>
+      <c r="I17" t="n">
+        <v>39552</v>
+      </c>
+      <c r="J17" t="n">
+        <v>45929</v>
+      </c>
+      <c r="K17" t="n">
+        <v>46478</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Europe (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>439.9</v>
+        <v>6863.27243246694</v>
       </c>
       <c r="D18" t="n">
-        <v>491.4</v>
+        <v>6963.91479812882</v>
       </c>
       <c r="E18" t="n">
-        <v>544.3</v>
+        <v>6979.49317509289</v>
       </c>
       <c r="F18" t="n">
-        <v>586.5</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+        <v>6988</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1625.1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1128.5</v>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -752,274 +787,80 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.9</v>
+        <v>31266.1315675331</v>
       </c>
       <c r="D19" t="n">
-        <v>2.1</v>
+        <v>31941.6092018712</v>
       </c>
       <c r="E19" t="n">
-        <v>2.2</v>
+        <v>32903.8678249071</v>
       </c>
       <c r="F19" t="n">
-        <v>2.4</v>
+        <v>33405</v>
       </c>
       <c r="G19" t="n">
-        <v>0.674</v>
+        <v>5968.8</v>
       </c>
       <c r="H19" t="n">
-        <v>1.236</v>
-      </c>
-      <c r="I19" t="n">
-        <v>2.471</v>
-      </c>
-      <c r="J19" t="n">
-        <v>2.955</v>
-      </c>
-      <c r="K19" t="n">
-        <v>3.195</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>South Asia (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="D20" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="E20" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="F20" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="G20" t="n">
-        <v>2.083</v>
-      </c>
-      <c r="H20" t="n">
-        <v>3.056</v>
-      </c>
-      <c r="I20" t="n">
-        <v>9.523</v>
-      </c>
-      <c r="J20" t="n">
-        <v>14.355</v>
-      </c>
-      <c r="K20" t="n">
-        <v>16.029</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Africa (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>262.6</v>
-      </c>
-      <c r="D21" t="n">
-        <v>271.2</v>
-      </c>
-      <c r="E21" t="n">
-        <v>272.5</v>
-      </c>
-      <c r="F21" t="n">
-        <v>284.2</v>
-      </c>
-      <c r="G21" t="n">
-        <v>73.902</v>
-      </c>
-      <c r="H21" t="n">
-        <v>62.351</v>
-      </c>
-      <c r="I21" t="n">
-        <v>195.241</v>
-      </c>
-      <c r="J21" t="n">
-        <v>234.123</v>
-      </c>
-      <c r="K21" t="n">
-        <v>252.546</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Americas (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>3508.5</v>
-      </c>
-      <c r="D22" t="n">
-        <v>3889.5</v>
-      </c>
-      <c r="E22" t="n">
-        <v>4084.7</v>
-      </c>
-      <c r="F22" t="n">
-        <v>4142</v>
-      </c>
-      <c r="G22" t="n">
-        <v>797.258</v>
-      </c>
-      <c r="H22" t="n">
-        <v>873.521</v>
-      </c>
-      <c r="I22" t="n">
-        <v>3045.921</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3800.781</v>
-      </c>
-      <c r="K22" t="n">
-        <v>4250.701</v>
-      </c>
+        <v>8046.4</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>3488.9</v>
-      </c>
-      <c r="D23" t="n">
-        <v>3888.7</v>
-      </c>
-      <c r="E23" t="n">
-        <v>3964.8</v>
-      </c>
-      <c r="F23" t="n">
-        <v>3962.6</v>
-      </c>
-      <c r="G23" t="n">
-        <v>579.165</v>
-      </c>
-      <c r="H23" t="n">
-        <v>313.499</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1202.564</v>
-      </c>
-      <c r="J23" t="n">
-        <v>2329.21</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2700.05</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Europe (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>26568.4</v>
-      </c>
-      <c r="D24" t="n">
-        <v>27635.3</v>
-      </c>
-      <c r="E24" t="n">
-        <v>28681.2</v>
-      </c>
-      <c r="F24" t="n">
-        <v>29489.2</v>
-      </c>
-      <c r="G24" t="n">
-        <v>10594.872</v>
-      </c>
-      <c r="H24" t="n">
-        <v>10047.669</v>
-      </c>
-      <c r="I24" t="n">
-        <v>23043.584</v>
-      </c>
-      <c r="J24" t="n">
-        <v>27129.43</v>
-      </c>
-      <c r="K24" t="n">
-        <v>28794.97</v>
+          <t>UN_Tourism_inbound_arrivals_by_region_12_2025</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>geo</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>series</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>673.1</v>
+        <v>2016</v>
       </c>
       <c r="D25" t="n">
-        <v>660.8</v>
+        <v>2017</v>
       </c>
       <c r="E25" t="n">
-        <v>636</v>
+        <v>2018</v>
       </c>
       <c r="F25" t="n">
-        <v>604.3</v>
+        <v>2019</v>
       </c>
       <c r="G25" t="n">
-        <v>95.996</v>
+        <v>2020</v>
       </c>
       <c r="H25" t="n">
-        <v>165.966</v>
+        <v>2021</v>
       </c>
       <c r="I25" t="n">
-        <v>404.707</v>
+        <v>2022</v>
       </c>
       <c r="J25" t="n">
-        <v>483.885</v>
+        <v>2023</v>
       </c>
       <c r="K25" t="n">
-        <v>489.689</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="26">
@@ -1030,230 +871,230 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>South Asia (UNWTO total)</t>
+          <t>Africa (UNWTO total)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>231.2</v>
+        <v>262.6</v>
       </c>
       <c r="D26" t="n">
-        <v>268.7</v>
+        <v>271.2</v>
       </c>
       <c r="E26" t="n">
-        <v>289.7</v>
+        <v>272.5</v>
       </c>
       <c r="F26" t="n">
-        <v>307.1</v>
+        <v>284.2</v>
       </c>
       <c r="G26" t="n">
-        <v>55.831</v>
+        <v>73.902</v>
       </c>
       <c r="H26" t="n">
-        <v>42.545</v>
+        <v>62.351</v>
       </c>
       <c r="I26" t="n">
-        <v>160.263</v>
+        <v>195.241</v>
       </c>
       <c r="J26" t="n">
-        <v>232.398</v>
+        <v>234.123</v>
       </c>
       <c r="K26" t="n">
-        <v>278.701</v>
+        <v>252.546</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Africa (UNWTO total)</t>
+          <t>Americas (UNWTO total)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1243</v>
+        <v>3508.5</v>
       </c>
       <c r="D27" t="n">
-        <v>1314.3</v>
+        <v>3889.5</v>
       </c>
       <c r="E27" t="n">
-        <v>1235.9</v>
+        <v>4084.7</v>
       </c>
       <c r="F27" t="n">
-        <v>1340</v>
+        <v>4142</v>
       </c>
       <c r="G27" t="n">
-        <v>262.945</v>
+        <v>797.258</v>
       </c>
       <c r="H27" t="n">
-        <v>250.284</v>
+        <v>873.521</v>
       </c>
       <c r="I27" t="n">
-        <v>830.221</v>
+        <v>3045.921</v>
       </c>
       <c r="J27" t="n">
-        <v>1025.13128294283</v>
+        <v>3800.781</v>
       </c>
       <c r="K27" t="n">
-        <v>1297.90576947888</v>
+        <v>4250.701</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Americas (UNWTO total)</t>
+          <t>East Asia and the Pacific (UNWTO total)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4573.9</v>
+        <v>3488.9</v>
       </c>
       <c r="D28" t="n">
-        <v>5866</v>
+        <v>3888.7</v>
       </c>
       <c r="E28" t="n">
-        <v>6370.5</v>
+        <v>3964.8</v>
       </c>
       <c r="F28" t="n">
-        <v>7092.1</v>
+        <v>3962.6</v>
       </c>
       <c r="G28" t="n">
-        <v>1320.48</v>
+        <v>579.165</v>
       </c>
       <c r="H28" t="n">
-        <v>1867.265</v>
+        <v>313.499</v>
       </c>
       <c r="I28" t="n">
-        <v>6359.413</v>
+        <v>1202.564</v>
       </c>
       <c r="J28" t="n">
-        <v>8470.624000010759</v>
+        <v>2329.21</v>
       </c>
       <c r="K28" t="n">
-        <v>9428.970904708071</v>
+        <v>2700.05</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>Europe (UNWTO total)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1904.7</v>
+        <v>26568.4</v>
       </c>
       <c r="D29" t="n">
-        <v>2299</v>
+        <v>27635.3</v>
       </c>
       <c r="E29" t="n">
-        <v>2560.7</v>
+        <v>28681.2</v>
       </c>
       <c r="F29" t="n">
-        <v>2977</v>
+        <v>29489.2</v>
       </c>
       <c r="G29" t="n">
-        <v>562.403</v>
+        <v>10594.872</v>
       </c>
       <c r="H29" t="n">
-        <v>230.302</v>
+        <v>10047.669</v>
       </c>
       <c r="I29" t="n">
-        <v>1086.684</v>
+        <v>23043.584</v>
       </c>
       <c r="J29" t="n">
-        <v>2360.18863897558</v>
+        <v>27129.43</v>
       </c>
       <c r="K29" t="n">
-        <v>2817.03795662791</v>
+        <v>28794.97</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Europe (UNWTO total)</t>
+          <t>Middle East (UNWTO total)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>67047.39999999999</v>
+        <v>673.1</v>
       </c>
       <c r="D30" t="n">
-        <v>71695.89999999999</v>
+        <v>660.8</v>
       </c>
       <c r="E30" t="n">
-        <v>71903.89999999999</v>
+        <v>636</v>
       </c>
       <c r="F30" t="n">
-        <v>71377.8</v>
+        <v>604.3</v>
       </c>
       <c r="G30" t="n">
-        <v>16676.276</v>
+        <v>95.996</v>
       </c>
       <c r="H30" t="n">
-        <v>28505.919</v>
+        <v>165.966</v>
       </c>
       <c r="I30" t="n">
-        <v>62765.346</v>
+        <v>404.707</v>
       </c>
       <c r="J30" t="n">
-        <v>72386.9099346476</v>
+        <v>483.885</v>
       </c>
       <c r="K30" t="n">
-        <v>79114.75530078731</v>
+        <v>489.689</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>South Asia (UNWTO total)</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>386.7</v>
+        <v>231.2</v>
       </c>
       <c r="D31" t="n">
-        <v>466.4</v>
+        <v>268.7</v>
       </c>
       <c r="E31" t="n">
-        <v>416.3</v>
+        <v>289.7</v>
       </c>
       <c r="F31" t="n">
-        <v>424.7</v>
+        <v>307.1</v>
       </c>
       <c r="G31" t="n">
-        <v>76.34399999999999</v>
+        <v>55.831</v>
       </c>
       <c r="H31" t="n">
-        <v>281.162</v>
+        <v>42.545</v>
       </c>
       <c r="I31" t="n">
-        <v>416.759</v>
+        <v>160.263</v>
       </c>
       <c r="J31" t="n">
-        <v>617.95432944935</v>
+        <v>232.398</v>
       </c>
       <c r="K31" t="n">
-        <v>765.914310277042</v>
+        <v>278.701</v>
       </c>
     </row>
     <row r="32">
@@ -1264,230 +1105,230 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>South Asia (UNWTO total)</t>
+          <t>Africa (UNWTO total)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>159.3</v>
+        <v>1243</v>
       </c>
       <c r="D32" t="n">
-        <v>227</v>
+        <v>1314.3</v>
       </c>
       <c r="E32" t="n">
-        <v>321</v>
+        <v>1235.9</v>
       </c>
       <c r="F32" t="n">
-        <v>297.5</v>
+        <v>1340</v>
       </c>
       <c r="G32" t="n">
-        <v>34.655</v>
+        <v>262.945</v>
       </c>
       <c r="H32" t="n">
-        <v>45.87</v>
+        <v>250.284</v>
       </c>
       <c r="I32" t="n">
-        <v>200.859</v>
+        <v>830.221</v>
       </c>
       <c r="J32" t="n">
-        <v>308.24178665693</v>
+        <v>1025.13128294283</v>
       </c>
       <c r="K32" t="n">
-        <v>334.712612593961</v>
+        <v>1297.90576947888</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Africa (UNWTO total)</t>
+          <t>Americas (UNWTO total)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>574.301</v>
+        <v>4573.9</v>
       </c>
       <c r="D33" t="n">
-        <v>585.447</v>
+        <v>5866</v>
       </c>
       <c r="E33" t="n">
-        <v>597.803</v>
+        <v>6370.5</v>
       </c>
       <c r="F33" t="n">
-        <v>566.6</v>
+        <v>7092.1</v>
       </c>
       <c r="G33" t="n">
-        <v>107.201</v>
+        <v>1320.48</v>
       </c>
       <c r="H33" t="n">
-        <v>153.671</v>
+        <v>1867.265</v>
       </c>
       <c r="I33" t="n">
-        <v>366.029</v>
+        <v>6359.413</v>
       </c>
       <c r="J33" t="n">
-        <v>529.515</v>
+        <v>8470.624000010759</v>
       </c>
       <c r="K33" t="n">
-        <v>586.16</v>
+        <v>9428.970904708071</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Americas (UNWTO total)</t>
+          <t>East Asia and the Pacific (UNWTO total)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>46459.207</v>
+        <v>1904.7</v>
       </c>
       <c r="D34" t="n">
-        <v>46675.98</v>
+        <v>2299</v>
       </c>
       <c r="E34" t="n">
-        <v>48966.068</v>
+        <v>2560.7</v>
       </c>
       <c r="F34" t="n">
-        <v>48061.7</v>
+        <v>2977</v>
       </c>
       <c r="G34" t="n">
-        <v>13952.619</v>
+        <v>562.403</v>
       </c>
       <c r="H34" t="n">
-        <v>18293.477</v>
+        <v>230.302</v>
       </c>
       <c r="I34" t="n">
-        <v>33573.32</v>
+        <v>1086.684</v>
       </c>
       <c r="J34" t="n">
-        <v>42840.828</v>
+        <v>2360.18863897558</v>
       </c>
       <c r="K34" t="n">
-        <v>46039.515</v>
+        <v>2817.03795662791</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>Europe (UNWTO total)</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>11764.684</v>
+        <v>67047.39999999999</v>
       </c>
       <c r="D35" t="n">
-        <v>12260.961</v>
+        <v>71695.89999999999</v>
       </c>
       <c r="E35" t="n">
-        <v>11952.945</v>
+        <v>71903.89999999999</v>
       </c>
       <c r="F35" t="n">
-        <v>12183.9</v>
+        <v>71377.8</v>
       </c>
       <c r="G35" t="n">
-        <v>2027.749</v>
+        <v>16676.276</v>
       </c>
       <c r="H35" t="n">
-        <v>816.227</v>
+        <v>28505.919</v>
       </c>
       <c r="I35" t="n">
-        <v>3455.282</v>
+        <v>62765.346</v>
       </c>
       <c r="J35" t="n">
-        <v>6726.311</v>
+        <v>72386.9099346476</v>
       </c>
       <c r="K35" t="n">
-        <v>7951.807</v>
+        <v>79114.75530078731</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Europe (UNWTO total)</t>
+          <t>Middle East (UNWTO total)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>15505.744</v>
+        <v>386.7</v>
       </c>
       <c r="D36" t="n">
-        <v>15633.303</v>
+        <v>466.4</v>
       </c>
       <c r="E36" t="n">
-        <v>16082.513</v>
+        <v>416.3</v>
       </c>
       <c r="F36" t="n">
-        <v>16381.9</v>
+        <v>424.7</v>
       </c>
       <c r="G36" t="n">
-        <v>2612.223</v>
+        <v>76.34399999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>2259.032</v>
+        <v>281.162</v>
       </c>
       <c r="I36" t="n">
-        <v>11567.835</v>
+        <v>416.759</v>
       </c>
       <c r="J36" t="n">
-        <v>13771.831</v>
+        <v>617.95432944935</v>
       </c>
       <c r="K36" t="n">
-        <v>14854.886</v>
+        <v>765.914310277042</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>South Asia (UNWTO total)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>681.191</v>
+        <v>159.3</v>
       </c>
       <c r="D37" t="n">
-        <v>550.013</v>
+        <v>227</v>
       </c>
       <c r="E37" t="n">
-        <v>576.227</v>
+        <v>321</v>
       </c>
       <c r="F37" t="n">
-        <v>577.1</v>
+        <v>297.5</v>
       </c>
       <c r="G37" t="n">
-        <v>127.276</v>
+        <v>34.655</v>
       </c>
       <c r="H37" t="n">
-        <v>227.801</v>
+        <v>45.87</v>
       </c>
       <c r="I37" t="n">
-        <v>366.673</v>
+        <v>200.859</v>
       </c>
       <c r="J37" t="n">
-        <v>463.179</v>
+        <v>308.24178665693</v>
       </c>
       <c r="K37" t="n">
-        <v>459.545</v>
+        <v>334.712612593961</v>
       </c>
     </row>
     <row r="38">
@@ -1498,36 +1339,647 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>574.301</v>
+      </c>
+      <c r="D38" t="n">
+        <v>585.447</v>
+      </c>
+      <c r="E38" t="n">
+        <v>597.803</v>
+      </c>
+      <c r="F38" t="n">
+        <v>566.6</v>
+      </c>
+      <c r="G38" t="n">
+        <v>107.201</v>
+      </c>
+      <c r="H38" t="n">
+        <v>153.671</v>
+      </c>
+      <c r="I38" t="n">
+        <v>366.029</v>
+      </c>
+      <c r="J38" t="n">
+        <v>529.515</v>
+      </c>
+      <c r="K38" t="n">
+        <v>586.16</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>46459.207</v>
+      </c>
+      <c r="D39" t="n">
+        <v>46675.98</v>
+      </c>
+      <c r="E39" t="n">
+        <v>48966.068</v>
+      </c>
+      <c r="F39" t="n">
+        <v>48061.7</v>
+      </c>
+      <c r="G39" t="n">
+        <v>13952.619</v>
+      </c>
+      <c r="H39" t="n">
+        <v>18293.477</v>
+      </c>
+      <c r="I39" t="n">
+        <v>33573.32</v>
+      </c>
+      <c r="J39" t="n">
+        <v>42840.828</v>
+      </c>
+      <c r="K39" t="n">
+        <v>46039.515</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>11764.684</v>
+      </c>
+      <c r="D40" t="n">
+        <v>12260.961</v>
+      </c>
+      <c r="E40" t="n">
+        <v>11952.945</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12183.9</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2027.749</v>
+      </c>
+      <c r="H40" t="n">
+        <v>816.227</v>
+      </c>
+      <c r="I40" t="n">
+        <v>3455.282</v>
+      </c>
+      <c r="J40" t="n">
+        <v>6726.311</v>
+      </c>
+      <c r="K40" t="n">
+        <v>7951.807</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>15505.744</v>
+      </c>
+      <c r="D41" t="n">
+        <v>15633.303</v>
+      </c>
+      <c r="E41" t="n">
+        <v>16082.513</v>
+      </c>
+      <c r="F41" t="n">
+        <v>16381.9</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2612.223</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2259.032</v>
+      </c>
+      <c r="I41" t="n">
+        <v>11567.835</v>
+      </c>
+      <c r="J41" t="n">
+        <v>13771.831</v>
+      </c>
+      <c r="K41" t="n">
+        <v>14854.886</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>681.191</v>
+      </c>
+      <c r="D42" t="n">
+        <v>550.013</v>
+      </c>
+      <c r="E42" t="n">
+        <v>576.227</v>
+      </c>
+      <c r="F42" t="n">
+        <v>577.1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>127.276</v>
+      </c>
+      <c r="H42" t="n">
+        <v>227.801</v>
+      </c>
+      <c r="I42" t="n">
+        <v>366.673</v>
+      </c>
+      <c r="J42" t="n">
+        <v>463.179</v>
+      </c>
+      <c r="K42" t="n">
+        <v>459.545</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>South Asia (UNWTO total)</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C43" t="n">
         <v>1422.361</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D43" t="n">
         <v>1481.042</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E43" t="n">
         <v>1570.362</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F43" t="n">
         <v>1670.5</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G43" t="n">
         <v>384.746</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H43" t="n">
         <v>528.2569999999999</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I43" t="n">
         <v>1440.26</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J43" t="n">
         <v>2016.472</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K43" t="n">
         <v>2496.501</v>
       </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_arrivals_by_transport_12_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G49" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H49" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I49" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K49" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>88747</v>
+      </c>
+      <c r="D50" t="n">
+        <v>94671</v>
+      </c>
+      <c r="E50" t="n">
+        <v>99763</v>
+      </c>
+      <c r="F50" t="n">
+        <v>102244</v>
+      </c>
+      <c r="G50" t="n">
+        <v>26432</v>
+      </c>
+      <c r="H50" t="n">
+        <v>34307</v>
+      </c>
+      <c r="I50" t="n">
+        <v>73226</v>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>6420</v>
+      </c>
+      <c r="D51" t="n">
+        <v>6635</v>
+      </c>
+      <c r="E51" t="n">
+        <v>6422</v>
+      </c>
+      <c r="F51" t="n">
+        <v>6684</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2412</v>
+      </c>
+      <c r="H51" t="n">
+        <v>3110</v>
+      </c>
+      <c r="I51" t="n">
+        <v>6028</v>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>60343.7</v>
+      </c>
+      <c r="D52" t="n">
+        <v>66639.5</v>
+      </c>
+      <c r="E52" t="n">
+        <v>67545.7</v>
+      </c>
+      <c r="F52" t="n">
+        <v>68691.89999999999</v>
+      </c>
+      <c r="G52" t="n">
+        <v>13657.664</v>
+      </c>
+      <c r="H52" t="n">
+        <v>24431.89</v>
+      </c>
+      <c r="I52" t="n">
+        <v>59307.849</v>
+      </c>
+      <c r="J52" t="n">
+        <v>69564.23140752919</v>
+      </c>
+      <c r="K52" t="n">
+        <v>77119.7871470598</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>13335.9</v>
+      </c>
+      <c r="D53" t="n">
+        <v>13263.4</v>
+      </c>
+      <c r="E53" t="n">
+        <v>13250.6</v>
+      </c>
+      <c r="F53" t="n">
+        <v>13096.5</v>
+      </c>
+      <c r="G53" t="n">
+        <v>5052.128</v>
+      </c>
+      <c r="H53" t="n">
+        <v>6521.955</v>
+      </c>
+      <c r="I53" t="n">
+        <v>11199.208</v>
+      </c>
+      <c r="J53" t="n">
+        <v>13745.4613453271</v>
+      </c>
+      <c r="K53" t="n">
+        <v>14535.4190698515</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1635.4</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1965.7</v>
+      </c>
+      <c r="E54" t="n">
+        <v>2012.1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1720.8</v>
+      </c>
+      <c r="G54" t="n">
+        <v>223.311</v>
+      </c>
+      <c r="H54" t="n">
+        <v>226.957</v>
+      </c>
+      <c r="I54" t="n">
+        <v>1152.225</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1859.35721985221</v>
+      </c>
+      <c r="K54" t="n">
+        <v>2104.09063755124</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>30483.8</v>
+      </c>
+      <c r="D55" t="n">
+        <v>34116.5</v>
+      </c>
+      <c r="E55" t="n">
+        <v>37229.5</v>
+      </c>
+      <c r="F55" t="n">
+        <v>39396.2</v>
+      </c>
+      <c r="G55" t="n">
+        <v>9277</v>
+      </c>
+      <c r="H55" t="n">
+        <v>10600</v>
+      </c>
+      <c r="I55" t="n">
+        <v>29042</v>
+      </c>
+      <c r="J55" t="n">
+        <v>35814</v>
+      </c>
+      <c r="K55" t="n">
+        <v>38587</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>1701.5</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1633.7</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1701</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1727.9</v>
+      </c>
+      <c r="G56" t="n">
+        <v>348</v>
+      </c>
+      <c r="H56" t="n">
+        <v>472</v>
+      </c>
+      <c r="I56" t="n">
+        <v>703</v>
+      </c>
+      <c r="J56" t="n">
+        <v>885</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>46940.691</v>
+      </c>
+      <c r="D57" t="n">
+        <v>48734.483</v>
+      </c>
+      <c r="E57" t="n">
+        <v>50695.476</v>
+      </c>
+      <c r="F57" t="n">
+        <v>50253.1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>10932.649</v>
+      </c>
+      <c r="H57" t="n">
+        <v>13735.582</v>
+      </c>
+      <c r="I57" t="n">
+        <v>31938.417</v>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>28913.34</v>
+      </c>
+      <c r="D58" t="n">
+        <v>27920.526</v>
+      </c>
+      <c r="E58" t="n">
+        <v>28489.235</v>
+      </c>
+      <c r="F58" t="n">
+        <v>28651.9</v>
+      </c>
+      <c r="G58" t="n">
+        <v>8221.689</v>
+      </c>
+      <c r="H58" t="n">
+        <v>8290.293</v>
+      </c>
+      <c r="I58" t="n">
+        <v>18383.956</v>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>553.457</v>
+      </c>
+      <c r="D59" t="n">
+        <v>531.737</v>
+      </c>
+      <c r="E59" t="n">
+        <v>561.207</v>
+      </c>
+      <c r="F59" t="n">
+        <v>536.7</v>
+      </c>
+      <c r="G59" t="n">
+        <v>57.676</v>
+      </c>
+      <c r="H59" t="n">
+        <v>74.578</v>
+      </c>
+      <c r="I59" t="n">
+        <v>547.312</v>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
framework tourism world 6/8
</commit_message>
<xml_diff>
--- a/outputs/world/views_single_sheet.xlsx
+++ b/outputs/world/views_single_sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,32 +450,40 @@
       <c r="H3" t="n">
         <v>2022</v>
       </c>
+      <c r="I3" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.99537</v>
+        <v>1.99315</v>
       </c>
       <c r="C4" t="n">
-        <v>3.9861</v>
+        <v>1.99379</v>
       </c>
       <c r="D4" t="n">
-        <v>3.97426</v>
+        <v>2.00237</v>
       </c>
       <c r="E4" t="n">
-        <v>3.85284</v>
+        <v>2.01469</v>
       </c>
       <c r="F4" t="n">
-        <v>2.35015</v>
+        <v>1.00336</v>
       </c>
       <c r="G4" t="n">
-        <v>2.16005</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+        <v>0.98237</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.41368</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.577</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -502,6 +510,7 @@
         <v>5.50139</v>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -520,196 +529,174 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8.4518</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8.487259999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.539569999999999</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8.61168</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6.76612</v>
+      </c>
+      <c r="G7" t="n">
+        <v>7.62444</v>
+      </c>
+      <c r="H7" t="n">
+        <v>8.462899999999999</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>2.88621</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C8" t="n">
         <v>2.9547</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>2.9604</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>3.01889</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F8" t="n">
         <v>2.1474</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G8" t="n">
         <v>2.76457</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H8" t="n">
         <v>2.96775</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>UN_Tourism_inbound_arrivals_by_purpose_12_2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>geo</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>series</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2016</v>
-      </c>
-      <c r="D13" t="n">
-        <v>2017</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2018</v>
-      </c>
-      <c r="F13" t="n">
-        <v>2019</v>
-      </c>
-      <c r="G13" t="n">
-        <v>2020</v>
-      </c>
-      <c r="H13" t="n">
-        <v>2021</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2022</v>
-      </c>
-      <c r="J13" t="n">
-        <v>2023</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2024</v>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_accommodation_12_2025</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>geo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
+          <t>series</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5703.7</v>
+        <v>2016</v>
       </c>
       <c r="D14" t="n">
-        <v>5706.7</v>
+        <v>2017</v>
       </c>
       <c r="E14" t="n">
-        <v>5636.8</v>
+        <v>2018</v>
       </c>
       <c r="F14" t="n">
-        <v>6112.7</v>
+        <v>2019</v>
       </c>
       <c r="G14" t="n">
-        <v>1565.465</v>
+        <v>2020</v>
       </c>
       <c r="H14" t="n">
-        <v>2270.304</v>
+        <v>2021</v>
       </c>
       <c r="I14" t="n">
-        <v>4952.511</v>
+        <v>2022</v>
       </c>
       <c r="J14" t="n">
-        <v>4973.06749958168</v>
+        <v>2023</v>
       </c>
       <c r="K14" t="n">
-        <v>5253.19541783694</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>69611.3</v>
-      </c>
-      <c r="D15" t="n">
-        <v>76161.7</v>
-      </c>
-      <c r="E15" t="n">
-        <v>77171.60000000001</v>
-      </c>
-      <c r="F15" t="n">
-        <v>77396.5</v>
-      </c>
-      <c r="G15" t="n">
-        <v>17367.6</v>
-      </c>
-      <c r="H15" t="n">
-        <v>28910.5</v>
-      </c>
-      <c r="I15" t="n">
-        <v>66706.8</v>
-      </c>
+          <t>inbound - accommodation - short-term accommodation, hotels and similar (ISIC 5510) - guests</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>80195.98247311771</v>
+        <v>7087</v>
       </c>
       <c r="K15" t="n">
-        <v>88506.1014367087</v>
+        <v>6612</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
+          <t>inbound - accommodation - short-term accommodation, hotels and similar (ISIC 5510) - guests</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14649</v>
+        <v>50297</v>
       </c>
       <c r="D16" t="n">
-        <v>14537</v>
+        <v>53334</v>
       </c>
       <c r="E16" t="n">
-        <v>14377.6</v>
+        <v>54146</v>
       </c>
       <c r="F16" t="n">
-        <v>14875.2</v>
+        <v>55982</v>
       </c>
       <c r="G16" t="n">
-        <v>6766</v>
+        <v>10894</v>
       </c>
       <c r="H16" t="n">
-        <v>8326</v>
+        <v>20451</v>
       </c>
       <c r="I16" t="n">
-        <v>10259</v>
+        <v>49568</v>
       </c>
       <c r="J16" t="n">
-        <v>11321</v>
+        <v>68632.25</v>
       </c>
       <c r="K16" t="n">
-        <v>11247</v>
+        <v>73766.842</v>
       </c>
     </row>
     <row r="17">
@@ -720,69 +707,75 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
+          <t>inbound - accommodation - short-term accommodation, hotels and similar (ISIC 5510) - guests</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>70275</v>
+        <v>43405</v>
       </c>
       <c r="D17" t="n">
-        <v>75394</v>
+        <v>45365</v>
       </c>
       <c r="E17" t="n">
-        <v>78850.89999999999</v>
+        <v>46825</v>
       </c>
       <c r="F17" t="n">
-        <v>80523.5</v>
+        <v>47377</v>
       </c>
       <c r="G17" t="n">
-        <v>18423</v>
+        <v>14387.445</v>
       </c>
       <c r="H17" t="n">
-        <v>18562</v>
+        <v>22915.817</v>
       </c>
       <c r="I17" t="n">
-        <v>39552</v>
+        <v>49193.898</v>
       </c>
       <c r="J17" t="n">
-        <v>45929</v>
+        <v>61506.242</v>
       </c>
       <c r="K17" t="n">
-        <v>46478</v>
+        <v>67311.56600000001</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
+          <t>inbound - accommodation - short-term accommodation, hotels and similar (ISIC 5510) - guests</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6863.27243246694</v>
+        <v>18875</v>
       </c>
       <c r="D18" t="n">
-        <v>6963.91479812882</v>
+        <v>21394</v>
       </c>
       <c r="E18" t="n">
-        <v>6979.49317509289</v>
+        <v>21764</v>
       </c>
       <c r="F18" t="n">
-        <v>6988</v>
+        <v>22614</v>
       </c>
       <c r="G18" t="n">
-        <v>1625.1</v>
+        <v>9556.136</v>
       </c>
       <c r="H18" t="n">
-        <v>1128.5</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+        <v>15267.289</v>
+      </c>
+      <c r="I18" t="n">
+        <v>21306.849</v>
+      </c>
+      <c r="J18" t="n">
+        <v>23167.132</v>
+      </c>
+      <c r="K18" t="n">
+        <v>23243.383</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -792,26 +785,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
+          <t>inbound - accommodation - short-term accommodation, hotels and similar (ISIC 5510) - guests</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>31266.1315675331</v>
+        <v>29588.417504</v>
       </c>
       <c r="D19" t="n">
-        <v>31941.6092018712</v>
+        <v>29802</v>
       </c>
       <c r="E19" t="n">
-        <v>32903.8678249071</v>
+        <v>30391</v>
       </c>
       <c r="F19" t="n">
-        <v>33405</v>
+        <v>30699</v>
       </c>
       <c r="G19" t="n">
-        <v>5968.8</v>
+        <v>5339</v>
       </c>
       <c r="H19" t="n">
-        <v>8046.4</v>
+        <v>4404</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -820,7 +813,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>UN_Tourism_inbound_arrivals_by_region_12_2025</t>
+          <t>UN_Tourism_inbound_arrivals_by_purpose_12_2025</t>
         </is>
       </c>
     </row>
@@ -866,820 +859,810 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Africa (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>262.6</v>
+        <v>16210.1</v>
       </c>
       <c r="D26" t="n">
-        <v>271.2</v>
+        <v>16793.1</v>
       </c>
       <c r="E26" t="n">
-        <v>272.5</v>
+        <v>17439</v>
       </c>
       <c r="F26" t="n">
-        <v>284.2</v>
-      </c>
-      <c r="G26" t="n">
-        <v>73.902</v>
-      </c>
-      <c r="H26" t="n">
-        <v>62.351</v>
-      </c>
-      <c r="I26" t="n">
-        <v>195.241</v>
-      </c>
+        <v>18260.8</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="n">
-        <v>234.123</v>
+        <v>16429</v>
       </c>
       <c r="K26" t="n">
-        <v>252.546</v>
+        <v>17963</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Americas (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3508.5</v>
+        <v>5703.7</v>
       </c>
       <c r="D27" t="n">
-        <v>3889.5</v>
+        <v>5706.7</v>
       </c>
       <c r="E27" t="n">
-        <v>4084.7</v>
+        <v>5636.8</v>
       </c>
       <c r="F27" t="n">
-        <v>4142</v>
+        <v>6112.7</v>
       </c>
       <c r="G27" t="n">
-        <v>797.258</v>
+        <v>1565.465</v>
       </c>
       <c r="H27" t="n">
-        <v>873.521</v>
+        <v>2270.304</v>
       </c>
       <c r="I27" t="n">
-        <v>3045.921</v>
+        <v>4952.511</v>
       </c>
       <c r="J27" t="n">
-        <v>3800.781</v>
+        <v>4973.06749958168</v>
       </c>
       <c r="K27" t="n">
-        <v>4250.701</v>
+        <v>5253.19541783694</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3488.9</v>
+        <v>69611.3</v>
       </c>
       <c r="D28" t="n">
-        <v>3888.7</v>
+        <v>76161.7</v>
       </c>
       <c r="E28" t="n">
-        <v>3964.8</v>
+        <v>77171.60000000001</v>
       </c>
       <c r="F28" t="n">
-        <v>3962.6</v>
+        <v>77396.5</v>
       </c>
       <c r="G28" t="n">
-        <v>579.165</v>
+        <v>17367.6</v>
       </c>
       <c r="H28" t="n">
-        <v>313.499</v>
+        <v>28910.5</v>
       </c>
       <c r="I28" t="n">
-        <v>1202.564</v>
+        <v>66706.8</v>
       </c>
       <c r="J28" t="n">
-        <v>2329.21</v>
+        <v>80195.98247311771</v>
       </c>
       <c r="K28" t="n">
-        <v>2700.05</v>
+        <v>88506.1014367087</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Europe (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>26568.4</v>
+        <v>14649</v>
       </c>
       <c r="D29" t="n">
-        <v>27635.3</v>
+        <v>14537</v>
       </c>
       <c r="E29" t="n">
-        <v>28681.2</v>
+        <v>14377.6</v>
       </c>
       <c r="F29" t="n">
-        <v>29489.2</v>
+        <v>14875.2</v>
       </c>
       <c r="G29" t="n">
-        <v>10594.872</v>
+        <v>6766</v>
       </c>
       <c r="H29" t="n">
-        <v>10047.669</v>
+        <v>8326</v>
       </c>
       <c r="I29" t="n">
-        <v>23043.584</v>
+        <v>10259</v>
       </c>
       <c r="J29" t="n">
-        <v>27129.43</v>
+        <v>11321</v>
       </c>
       <c r="K29" t="n">
-        <v>28794.97</v>
+        <v>11247</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>673.1</v>
+        <v>70275</v>
       </c>
       <c r="D30" t="n">
-        <v>660.8</v>
+        <v>75394</v>
       </c>
       <c r="E30" t="n">
-        <v>636</v>
+        <v>78850.89999999999</v>
       </c>
       <c r="F30" t="n">
-        <v>604.3</v>
+        <v>80523.5</v>
       </c>
       <c r="G30" t="n">
-        <v>95.996</v>
+        <v>18423</v>
       </c>
       <c r="H30" t="n">
-        <v>165.966</v>
+        <v>18562</v>
       </c>
       <c r="I30" t="n">
-        <v>404.707</v>
+        <v>39552</v>
       </c>
       <c r="J30" t="n">
-        <v>483.885</v>
+        <v>45929</v>
       </c>
       <c r="K30" t="n">
-        <v>489.689</v>
+        <v>46478</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>South Asia (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>231.2</v>
+        <v>1628</v>
       </c>
       <c r="D31" t="n">
-        <v>268.7</v>
+        <v>1935.7</v>
       </c>
       <c r="E31" t="n">
-        <v>289.7</v>
+        <v>2002.4</v>
       </c>
       <c r="F31" t="n">
-        <v>307.1</v>
+        <v>1890.7</v>
       </c>
       <c r="G31" t="n">
-        <v>55.831</v>
+        <v>498.255</v>
       </c>
       <c r="H31" t="n">
-        <v>42.545</v>
+        <v>573.603</v>
       </c>
       <c r="I31" t="n">
-        <v>160.263</v>
+        <v>1142.118</v>
       </c>
       <c r="J31" t="n">
-        <v>232.398</v>
+        <v>1326</v>
       </c>
       <c r="K31" t="n">
-        <v>278.701</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Africa (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1243</v>
+        <v>33451</v>
       </c>
       <c r="D32" t="n">
-        <v>1314.3</v>
+        <v>37355.3</v>
       </c>
       <c r="E32" t="n">
-        <v>1235.9</v>
+        <v>39310.3</v>
       </c>
       <c r="F32" t="n">
-        <v>1340</v>
+        <v>43133.7</v>
       </c>
       <c r="G32" t="n">
-        <v>262.945</v>
+        <v>23785.3</v>
       </c>
       <c r="H32" t="n">
-        <v>250.284</v>
+        <v>31286.8</v>
       </c>
       <c r="I32" t="n">
-        <v>830.221</v>
+        <v>37183.4</v>
       </c>
       <c r="J32" t="n">
-        <v>1025.13128294283</v>
+        <v>41926</v>
       </c>
       <c r="K32" t="n">
-        <v>1297.90576947888</v>
+        <v>46053</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Americas (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_BNSS_TOUR</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4573.9</v>
+        <v>6863.27243246694</v>
       </c>
       <c r="D33" t="n">
-        <v>5866</v>
+        <v>6963.91479812882</v>
       </c>
       <c r="E33" t="n">
-        <v>6370.5</v>
+        <v>6979.49317509289</v>
       </c>
       <c r="F33" t="n">
-        <v>7092.1</v>
+        <v>6988</v>
       </c>
       <c r="G33" t="n">
-        <v>1320.48</v>
+        <v>1625.1</v>
       </c>
       <c r="H33" t="n">
-        <v>1867.265</v>
-      </c>
-      <c r="I33" t="n">
-        <v>6359.413</v>
-      </c>
-      <c r="J33" t="n">
-        <v>8470.624000010759</v>
-      </c>
-      <c r="K33" t="n">
-        <v>9428.970904708071</v>
-      </c>
+        <v>1128.5</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>INBD_TRIP_PRPS_PERS_TOUR</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1904.7</v>
+        <v>31266.1315675331</v>
       </c>
       <c r="D34" t="n">
-        <v>2299</v>
+        <v>31941.6092018712</v>
       </c>
       <c r="E34" t="n">
-        <v>2560.7</v>
+        <v>32903.8678249071</v>
       </c>
       <c r="F34" t="n">
-        <v>2977</v>
+        <v>33405</v>
       </c>
       <c r="G34" t="n">
-        <v>562.403</v>
+        <v>5968.8</v>
       </c>
       <c r="H34" t="n">
-        <v>230.302</v>
-      </c>
-      <c r="I34" t="n">
-        <v>1086.684</v>
-      </c>
-      <c r="J34" t="n">
-        <v>2360.18863897558</v>
-      </c>
-      <c r="K34" t="n">
-        <v>2817.03795662791</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Europe (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>67047.39999999999</v>
-      </c>
-      <c r="D35" t="n">
-        <v>71695.89999999999</v>
-      </c>
-      <c r="E35" t="n">
-        <v>71903.89999999999</v>
-      </c>
-      <c r="F35" t="n">
-        <v>71377.8</v>
-      </c>
-      <c r="G35" t="n">
-        <v>16676.276</v>
-      </c>
-      <c r="H35" t="n">
-        <v>28505.919</v>
-      </c>
-      <c r="I35" t="n">
-        <v>62765.346</v>
-      </c>
-      <c r="J35" t="n">
-        <v>72386.9099346476</v>
-      </c>
-      <c r="K35" t="n">
-        <v>79114.75530078731</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Middle East (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>386.7</v>
-      </c>
-      <c r="D36" t="n">
-        <v>466.4</v>
-      </c>
-      <c r="E36" t="n">
-        <v>416.3</v>
-      </c>
-      <c r="F36" t="n">
-        <v>424.7</v>
-      </c>
-      <c r="G36" t="n">
-        <v>76.34399999999999</v>
-      </c>
-      <c r="H36" t="n">
-        <v>281.162</v>
-      </c>
-      <c r="I36" t="n">
-        <v>416.759</v>
-      </c>
-      <c r="J36" t="n">
-        <v>617.95432944935</v>
-      </c>
-      <c r="K36" t="n">
-        <v>765.914310277042</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>South Asia (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>159.3</v>
-      </c>
-      <c r="D37" t="n">
-        <v>227</v>
-      </c>
-      <c r="E37" t="n">
-        <v>321</v>
-      </c>
-      <c r="F37" t="n">
-        <v>297.5</v>
-      </c>
-      <c r="G37" t="n">
-        <v>34.655</v>
-      </c>
-      <c r="H37" t="n">
-        <v>45.87</v>
-      </c>
-      <c r="I37" t="n">
-        <v>200.859</v>
-      </c>
-      <c r="J37" t="n">
-        <v>308.24178665693</v>
-      </c>
-      <c r="K37" t="n">
-        <v>334.712612593961</v>
-      </c>
+        <v>8046.4</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Africa (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>574.301</v>
-      </c>
-      <c r="D38" t="n">
-        <v>585.447</v>
-      </c>
-      <c r="E38" t="n">
-        <v>597.803</v>
-      </c>
-      <c r="F38" t="n">
-        <v>566.6</v>
-      </c>
-      <c r="G38" t="n">
-        <v>107.201</v>
-      </c>
-      <c r="H38" t="n">
-        <v>153.671</v>
-      </c>
-      <c r="I38" t="n">
-        <v>366.029</v>
-      </c>
-      <c r="J38" t="n">
-        <v>529.515</v>
-      </c>
-      <c r="K38" t="n">
-        <v>586.16</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Americas (UNWTO total)</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>46459.207</v>
-      </c>
-      <c r="D39" t="n">
-        <v>46675.98</v>
-      </c>
-      <c r="E39" t="n">
-        <v>48966.068</v>
-      </c>
-      <c r="F39" t="n">
-        <v>48061.7</v>
-      </c>
-      <c r="G39" t="n">
-        <v>13952.619</v>
-      </c>
-      <c r="H39" t="n">
-        <v>18293.477</v>
-      </c>
-      <c r="I39" t="n">
-        <v>33573.32</v>
-      </c>
-      <c r="J39" t="n">
-        <v>42840.828</v>
-      </c>
-      <c r="K39" t="n">
-        <v>46039.515</v>
+          <t>UN_Tourism_inbound_arrivals_by_region_12_2025</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>geo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>East Asia and the Pacific (UNWTO total)</t>
+          <t>series</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>11764.684</v>
+        <v>2016</v>
       </c>
       <c r="D40" t="n">
-        <v>12260.961</v>
+        <v>2017</v>
       </c>
       <c r="E40" t="n">
-        <v>11952.945</v>
+        <v>2018</v>
       </c>
       <c r="F40" t="n">
-        <v>12183.9</v>
+        <v>2019</v>
       </c>
       <c r="G40" t="n">
-        <v>2027.749</v>
+        <v>2020</v>
       </c>
       <c r="H40" t="n">
-        <v>816.227</v>
+        <v>2021</v>
       </c>
       <c r="I40" t="n">
-        <v>3455.282</v>
+        <v>2022</v>
       </c>
       <c r="J40" t="n">
-        <v>6726.311</v>
+        <v>2023</v>
       </c>
       <c r="K40" t="n">
-        <v>7951.807</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Europe (UNWTO total)</t>
+          <t>Africa (UNWTO total)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>15505.744</v>
+        <v>124.1</v>
       </c>
       <c r="D41" t="n">
-        <v>15633.303</v>
+        <v>132.5</v>
       </c>
       <c r="E41" t="n">
-        <v>16082.513</v>
+        <v>143.4</v>
       </c>
       <c r="F41" t="n">
-        <v>16381.9</v>
+        <v>165.5</v>
       </c>
       <c r="G41" t="n">
-        <v>2612.223</v>
+        <v>30</v>
       </c>
       <c r="H41" t="n">
-        <v>2259.032</v>
+        <v>39</v>
       </c>
       <c r="I41" t="n">
-        <v>11567.835</v>
+        <v>112</v>
       </c>
       <c r="J41" t="n">
-        <v>13771.831</v>
+        <v>216</v>
       </c>
       <c r="K41" t="n">
-        <v>14854.886</v>
+        <v>235</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Middle East (UNWTO total)</t>
+          <t>Americas (UNWTO total)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>681.191</v>
+        <v>14587.7</v>
       </c>
       <c r="D42" t="n">
-        <v>550.013</v>
+        <v>15150</v>
       </c>
       <c r="E42" t="n">
-        <v>576.227</v>
+        <v>15405.4</v>
       </c>
       <c r="F42" t="n">
-        <v>577.1</v>
+        <v>16085</v>
       </c>
       <c r="G42" t="n">
-        <v>127.276</v>
+        <v>2130</v>
       </c>
       <c r="H42" t="n">
-        <v>227.801</v>
+        <v>2280</v>
       </c>
       <c r="I42" t="n">
-        <v>366.673</v>
+        <v>9776</v>
       </c>
       <c r="J42" t="n">
-        <v>463.179</v>
+        <v>13859</v>
       </c>
       <c r="K42" t="n">
-        <v>459.545</v>
+        <v>15051</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1994</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2182.5</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2149.3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2176.2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>299</v>
+      </c>
+      <c r="H43" t="n">
+        <v>129</v>
+      </c>
+      <c r="I43" t="n">
+        <v>567</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1154</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2875.8</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2974.9</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2943.9</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3150.3</v>
+      </c>
+      <c r="G44" t="n">
+        <v>392</v>
+      </c>
+      <c r="H44" t="n">
+        <v>460</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1998</v>
+      </c>
+      <c r="J44" t="n">
+        <v>2503</v>
+      </c>
+      <c r="K44" t="n">
+        <v>2624</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>116.1</v>
+      </c>
+      <c r="E45" t="n">
+        <v>110.1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>121</v>
+      </c>
+      <c r="G45" t="n">
+        <v>26</v>
+      </c>
+      <c r="H45" t="n">
+        <v>40</v>
+      </c>
+      <c r="I45" t="n">
+        <v>76</v>
+      </c>
+      <c r="J45" t="n">
+        <v>111</v>
+      </c>
+      <c r="K45" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>South Asia (UNWTO total)</t>
         </is>
       </c>
-      <c r="C43" t="n">
-        <v>1422.361</v>
-      </c>
-      <c r="D43" t="n">
-        <v>1481.042</v>
-      </c>
-      <c r="E43" t="n">
-        <v>1570.362</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1670.5</v>
-      </c>
-      <c r="G43" t="n">
-        <v>384.746</v>
-      </c>
-      <c r="H43" t="n">
-        <v>528.2569999999999</v>
-      </c>
-      <c r="I43" t="n">
-        <v>1440.26</v>
-      </c>
-      <c r="J43" t="n">
-        <v>2016.472</v>
-      </c>
-      <c r="K43" t="n">
-        <v>2496.501</v>
+      <c r="C46" t="n">
+        <v>274.2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>327.1</v>
+      </c>
+      <c r="E46" t="n">
+        <v>380.6</v>
+      </c>
+      <c r="F46" t="n">
+        <v>446.8</v>
+      </c>
+      <c r="G46" t="n">
+        <v>84</v>
+      </c>
+      <c r="H46" t="n">
+        <v>114</v>
+      </c>
+      <c r="I46" t="n">
+        <v>295</v>
+      </c>
+      <c r="J46" t="n">
+        <v>502</v>
+      </c>
+      <c r="K46" t="n">
+        <v>523</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>UN_Tourism_inbound_arrivals_by_transport_12_2025</t>
-        </is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1243</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1314.3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1235.9</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1340</v>
+      </c>
+      <c r="G47" t="n">
+        <v>262.945</v>
+      </c>
+      <c r="H47" t="n">
+        <v>250.284</v>
+      </c>
+      <c r="I47" t="n">
+        <v>830.221</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1025.13128294283</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1297.90576947888</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4573.9</v>
+      </c>
+      <c r="D48" t="n">
+        <v>5866</v>
+      </c>
+      <c r="E48" t="n">
+        <v>6370.5</v>
+      </c>
+      <c r="F48" t="n">
+        <v>7092.1</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1320.48</v>
+      </c>
+      <c r="H48" t="n">
+        <v>1867.265</v>
+      </c>
+      <c r="I48" t="n">
+        <v>6359.413</v>
+      </c>
+      <c r="J48" t="n">
+        <v>8470.624000010759</v>
+      </c>
+      <c r="K48" t="n">
+        <v>9428.970904708071</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>geo</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>series</t>
+          <t>East Asia and the Pacific (UNWTO total)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2016</v>
+        <v>1904.7</v>
       </c>
       <c r="D49" t="n">
-        <v>2017</v>
+        <v>2299</v>
       </c>
       <c r="E49" t="n">
-        <v>2018</v>
+        <v>2560.7</v>
       </c>
       <c r="F49" t="n">
-        <v>2019</v>
+        <v>2977</v>
       </c>
       <c r="G49" t="n">
-        <v>2020</v>
+        <v>562.403</v>
       </c>
       <c r="H49" t="n">
-        <v>2021</v>
+        <v>230.302</v>
       </c>
       <c r="I49" t="n">
-        <v>2022</v>
+        <v>1086.684</v>
       </c>
       <c r="J49" t="n">
-        <v>2023</v>
+        <v>2360.18863897558</v>
       </c>
       <c r="K49" t="n">
-        <v>2024</v>
+        <v>2817.03795662791</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+          <t>Europe (UNWTO total)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>88747</v>
+        <v>67047.39999999999</v>
       </c>
       <c r="D50" t="n">
-        <v>94671</v>
+        <v>71695.89999999999</v>
       </c>
       <c r="E50" t="n">
-        <v>99763</v>
+        <v>71903.89999999999</v>
       </c>
       <c r="F50" t="n">
-        <v>102244</v>
+        <v>71377.8</v>
       </c>
       <c r="G50" t="n">
-        <v>26432</v>
+        <v>16676.276</v>
       </c>
       <c r="H50" t="n">
-        <v>34307</v>
+        <v>28505.919</v>
       </c>
       <c r="I50" t="n">
-        <v>73226</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
+        <v>62765.346</v>
+      </c>
+      <c r="J50" t="n">
+        <v>72386.9099346476</v>
+      </c>
+      <c r="K50" t="n">
+        <v>79114.75530078731</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+          <t>Middle East (UNWTO total)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6420</v>
+        <v>386.7</v>
       </c>
       <c r="D51" t="n">
-        <v>6635</v>
+        <v>466.4</v>
       </c>
       <c r="E51" t="n">
-        <v>6422</v>
+        <v>416.3</v>
       </c>
       <c r="F51" t="n">
-        <v>6684</v>
+        <v>424.7</v>
       </c>
       <c r="G51" t="n">
-        <v>2412</v>
+        <v>76.34399999999999</v>
       </c>
       <c r="H51" t="n">
-        <v>3110</v>
+        <v>281.162</v>
       </c>
       <c r="I51" t="n">
-        <v>6028</v>
-      </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
+        <v>416.759</v>
+      </c>
+      <c r="J51" t="n">
+        <v>617.95432944935</v>
+      </c>
+      <c r="K51" t="n">
+        <v>765.914310277042</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1689,262 +1672,270 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+          <t>South Asia (UNWTO total)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>60343.7</v>
+        <v>159.3</v>
       </c>
       <c r="D52" t="n">
-        <v>66639.5</v>
+        <v>227</v>
       </c>
       <c r="E52" t="n">
-        <v>67545.7</v>
+        <v>321</v>
       </c>
       <c r="F52" t="n">
-        <v>68691.89999999999</v>
+        <v>297.5</v>
       </c>
       <c r="G52" t="n">
-        <v>13657.664</v>
+        <v>34.655</v>
       </c>
       <c r="H52" t="n">
-        <v>24431.89</v>
+        <v>45.87</v>
       </c>
       <c r="I52" t="n">
-        <v>59307.849</v>
+        <v>200.859</v>
       </c>
       <c r="J52" t="n">
-        <v>69564.23140752919</v>
+        <v>308.24178665693</v>
       </c>
       <c r="K52" t="n">
-        <v>77119.7871470598</v>
+        <v>334.712612593961</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+          <t>Africa (UNWTO total)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>13335.9</v>
+        <v>25.6</v>
       </c>
       <c r="D53" t="n">
-        <v>13263.4</v>
+        <v>27.6</v>
       </c>
       <c r="E53" t="n">
-        <v>13250.6</v>
+        <v>32.7</v>
       </c>
       <c r="F53" t="n">
-        <v>13096.5</v>
+        <v>33.6</v>
       </c>
       <c r="G53" t="n">
-        <v>5052.128</v>
+        <v>8.821999999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>6521.955</v>
+        <v>14.051</v>
       </c>
       <c r="I53" t="n">
-        <v>11199.208</v>
+        <v>25.231</v>
       </c>
       <c r="J53" t="n">
-        <v>13745.4613453271</v>
+        <v>25.175</v>
       </c>
       <c r="K53" t="n">
-        <v>14535.4190698515</v>
+        <v>24.723</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+          <t>Americas (UNWTO total)</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1635.4</v>
+        <v>31490.2</v>
       </c>
       <c r="D54" t="n">
-        <v>1965.7</v>
+        <v>35340.2</v>
       </c>
       <c r="E54" t="n">
-        <v>2012.1</v>
+        <v>38247.9</v>
       </c>
       <c r="F54" t="n">
-        <v>1720.8</v>
+        <v>41938.6</v>
       </c>
       <c r="G54" t="n">
-        <v>223.311</v>
+        <v>6980.967</v>
       </c>
       <c r="H54" t="n">
-        <v>226.957</v>
+        <v>12505.975</v>
       </c>
       <c r="I54" t="n">
-        <v>1152.225</v>
+        <v>17575.432</v>
       </c>
       <c r="J54" t="n">
-        <v>1859.35721985221</v>
+        <v>17057.584</v>
       </c>
       <c r="K54" t="n">
-        <v>2104.09063755124</v>
+        <v>18253.981</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+          <t>East Asia and the Pacific (UNWTO total)</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>30483.8</v>
+        <v>370.1</v>
       </c>
       <c r="D55" t="n">
-        <v>34116.5</v>
+        <v>411.6</v>
       </c>
       <c r="E55" t="n">
-        <v>37229.5</v>
+        <v>437.4</v>
       </c>
       <c r="F55" t="n">
-        <v>39396.2</v>
+        <v>437.2</v>
       </c>
       <c r="G55" t="n">
-        <v>9277</v>
+        <v>102.894</v>
       </c>
       <c r="H55" t="n">
-        <v>10600</v>
+        <v>54.699</v>
       </c>
       <c r="I55" t="n">
-        <v>29042</v>
+        <v>142.697</v>
       </c>
       <c r="J55" t="n">
-        <v>35814</v>
+        <v>257.555</v>
       </c>
       <c r="K55" t="n">
-        <v>38587</v>
+        <v>312.311</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+          <t>Europe (UNWTO total)</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1701.5</v>
+        <v>1832.9</v>
       </c>
       <c r="D56" t="n">
-        <v>1633.7</v>
+        <v>1961.7</v>
       </c>
       <c r="E56" t="n">
-        <v>1701</v>
+        <v>2056.6</v>
       </c>
       <c r="F56" t="n">
-        <v>1727.9</v>
+        <v>2105.1</v>
       </c>
       <c r="G56" t="n">
-        <v>348</v>
+        <v>559.011</v>
       </c>
       <c r="H56" t="n">
-        <v>472</v>
+        <v>963.153</v>
       </c>
       <c r="I56" t="n">
-        <v>703</v>
+        <v>2103.138</v>
       </c>
       <c r="J56" t="n">
-        <v>885</v>
+        <v>1938.865</v>
       </c>
       <c r="K56" t="n">
-        <v>1275</v>
+        <v>1788.665</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+          <t>Middle East (UNWTO total)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>46940.691</v>
+        <v>45.8</v>
       </c>
       <c r="D57" t="n">
-        <v>48734.483</v>
+        <v>50</v>
       </c>
       <c r="E57" t="n">
-        <v>50695.476</v>
+        <v>61</v>
       </c>
       <c r="F57" t="n">
-        <v>50253.1</v>
+        <v>53.8</v>
       </c>
       <c r="G57" t="n">
-        <v>10932.649</v>
+        <v>27.265</v>
       </c>
       <c r="H57" t="n">
-        <v>13735.582</v>
+        <v>77.745</v>
       </c>
       <c r="I57" t="n">
-        <v>31938.417</v>
-      </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+        <v>94.98</v>
+      </c>
+      <c r="J57" t="n">
+        <v>81.999</v>
+      </c>
+      <c r="K57" t="n">
+        <v>70.41</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+          <t>South Asia (UNWTO total)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>28913.34</v>
+        <v>23.9</v>
       </c>
       <c r="D58" t="n">
-        <v>27920.526</v>
+        <v>26.3</v>
       </c>
       <c r="E58" t="n">
-        <v>28489.235</v>
+        <v>32.4</v>
       </c>
       <c r="F58" t="n">
-        <v>28651.9</v>
+        <v>33</v>
       </c>
       <c r="G58" t="n">
-        <v>8221.689</v>
+        <v>7.483</v>
       </c>
       <c r="H58" t="n">
-        <v>8290.293</v>
+        <v>44.228</v>
       </c>
       <c r="I58" t="n">
-        <v>18383.956</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+        <v>40.493</v>
+      </c>
+      <c r="J58" t="n">
+        <v>45.088</v>
+      </c>
+      <c r="K58" t="n">
+        <v>40.784</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1954,32 +1945,997 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>Africa (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>574.301</v>
+      </c>
+      <c r="D59" t="n">
+        <v>585.447</v>
+      </c>
+      <c r="E59" t="n">
+        <v>597.803</v>
+      </c>
+      <c r="F59" t="n">
+        <v>566.6</v>
+      </c>
+      <c r="G59" t="n">
+        <v>107.201</v>
+      </c>
+      <c r="H59" t="n">
+        <v>153.671</v>
+      </c>
+      <c r="I59" t="n">
+        <v>366.029</v>
+      </c>
+      <c r="J59" t="n">
+        <v>529.515</v>
+      </c>
+      <c r="K59" t="n">
+        <v>586.16</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Americas (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>46459.207</v>
+      </c>
+      <c r="D60" t="n">
+        <v>46675.98</v>
+      </c>
+      <c r="E60" t="n">
+        <v>48966.068</v>
+      </c>
+      <c r="F60" t="n">
+        <v>48061.7</v>
+      </c>
+      <c r="G60" t="n">
+        <v>13952.619</v>
+      </c>
+      <c r="H60" t="n">
+        <v>18293.477</v>
+      </c>
+      <c r="I60" t="n">
+        <v>33573.32</v>
+      </c>
+      <c r="J60" t="n">
+        <v>42840.828</v>
+      </c>
+      <c r="K60" t="n">
+        <v>46039.515</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>East Asia and the Pacific (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>11764.684</v>
+      </c>
+      <c r="D61" t="n">
+        <v>12260.961</v>
+      </c>
+      <c r="E61" t="n">
+        <v>11952.945</v>
+      </c>
+      <c r="F61" t="n">
+        <v>12183.9</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2027.749</v>
+      </c>
+      <c r="H61" t="n">
+        <v>816.227</v>
+      </c>
+      <c r="I61" t="n">
+        <v>3455.282</v>
+      </c>
+      <c r="J61" t="n">
+        <v>6726.311</v>
+      </c>
+      <c r="K61" t="n">
+        <v>7951.807</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Europe (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>15505.744</v>
+      </c>
+      <c r="D62" t="n">
+        <v>15633.303</v>
+      </c>
+      <c r="E62" t="n">
+        <v>16082.513</v>
+      </c>
+      <c r="F62" t="n">
+        <v>16381.9</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2612.223</v>
+      </c>
+      <c r="H62" t="n">
+        <v>2259.032</v>
+      </c>
+      <c r="I62" t="n">
+        <v>11567.835</v>
+      </c>
+      <c r="J62" t="n">
+        <v>13771.831</v>
+      </c>
+      <c r="K62" t="n">
+        <v>14854.886</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Middle East (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>681.191</v>
+      </c>
+      <c r="D63" t="n">
+        <v>550.013</v>
+      </c>
+      <c r="E63" t="n">
+        <v>576.227</v>
+      </c>
+      <c r="F63" t="n">
+        <v>577.1</v>
+      </c>
+      <c r="G63" t="n">
+        <v>127.276</v>
+      </c>
+      <c r="H63" t="n">
+        <v>227.801</v>
+      </c>
+      <c r="I63" t="n">
+        <v>366.673</v>
+      </c>
+      <c r="J63" t="n">
+        <v>463.179</v>
+      </c>
+      <c r="K63" t="n">
+        <v>459.545</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>South Asia (UNWTO total)</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>1422.361</v>
+      </c>
+      <c r="D64" t="n">
+        <v>1481.042</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1570.362</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1670.5</v>
+      </c>
+      <c r="G64" t="n">
+        <v>384.746</v>
+      </c>
+      <c r="H64" t="n">
+        <v>528.2569999999999</v>
+      </c>
+      <c r="I64" t="n">
+        <v>1440.26</v>
+      </c>
+      <c r="J64" t="n">
+        <v>2016.472</v>
+      </c>
+      <c r="K64" t="n">
+        <v>2496.501</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_arrivals_by_transport_12_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D70" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E70" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F70" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G70" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H70" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I70" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J70" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K70" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>9802.4</v>
+      </c>
+      <c r="D71" t="n">
+        <v>10576.8</v>
+      </c>
+      <c r="E71" t="n">
+        <v>10372.1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>10999</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1664</v>
+      </c>
+      <c r="H71" t="n">
+        <v>1595</v>
+      </c>
+      <c r="I71" t="n">
+        <v>6669</v>
+      </c>
+      <c r="J71" t="n">
+        <v>9364</v>
+      </c>
+      <c r="K71" t="n">
+        <v>10269</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>9373.4</v>
+      </c>
+      <c r="D72" t="n">
+        <v>9458.5</v>
+      </c>
+      <c r="E72" t="n">
+        <v>9802.299999999999</v>
+      </c>
+      <c r="F72" t="n">
+        <v>10032.9</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1294</v>
+      </c>
+      <c r="H72" t="n">
+        <v>1461</v>
+      </c>
+      <c r="I72" t="n">
+        <v>5767</v>
+      </c>
+      <c r="J72" t="n">
+        <v>8449</v>
+      </c>
+      <c r="K72" t="n">
+        <v>9142</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
         </is>
       </c>
-      <c r="C59" t="n">
+      <c r="C73" t="n">
+        <v>795.5</v>
+      </c>
+      <c r="D73" t="n">
+        <v>847.9</v>
+      </c>
+      <c r="E73" t="n">
+        <v>959.5</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1113.5</v>
+      </c>
+      <c r="G73" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" t="n">
+        <v>6</v>
+      </c>
+      <c r="I73" t="n">
+        <v>388</v>
+      </c>
+      <c r="J73" t="n">
+        <v>531</v>
+      </c>
+      <c r="K73" t="n">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>60343.7</v>
+      </c>
+      <c r="D74" t="n">
+        <v>66639.5</v>
+      </c>
+      <c r="E74" t="n">
+        <v>67545.7</v>
+      </c>
+      <c r="F74" t="n">
+        <v>68691.89999999999</v>
+      </c>
+      <c r="G74" t="n">
+        <v>13657.664</v>
+      </c>
+      <c r="H74" t="n">
+        <v>24431.89</v>
+      </c>
+      <c r="I74" t="n">
+        <v>59307.849</v>
+      </c>
+      <c r="J74" t="n">
+        <v>69564.23140752919</v>
+      </c>
+      <c r="K74" t="n">
+        <v>77119.7871470598</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>13335.9</v>
+      </c>
+      <c r="D75" t="n">
+        <v>13263.4</v>
+      </c>
+      <c r="E75" t="n">
+        <v>13250.6</v>
+      </c>
+      <c r="F75" t="n">
+        <v>13096.5</v>
+      </c>
+      <c r="G75" t="n">
+        <v>5052.128</v>
+      </c>
+      <c r="H75" t="n">
+        <v>6521.955</v>
+      </c>
+      <c r="I75" t="n">
+        <v>11199.208</v>
+      </c>
+      <c r="J75" t="n">
+        <v>13745.4613453271</v>
+      </c>
+      <c r="K75" t="n">
+        <v>14535.4190698515</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1635.4</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1965.7</v>
+      </c>
+      <c r="E76" t="n">
+        <v>2012.1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>1720.8</v>
+      </c>
+      <c r="G76" t="n">
+        <v>223.311</v>
+      </c>
+      <c r="H76" t="n">
+        <v>226.957</v>
+      </c>
+      <c r="I76" t="n">
+        <v>1152.225</v>
+      </c>
+      <c r="J76" t="n">
+        <v>1859.35721985221</v>
+      </c>
+      <c r="K76" t="n">
+        <v>2104.09063755124</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>30483.8</v>
+      </c>
+      <c r="D77" t="n">
+        <v>34116.5</v>
+      </c>
+      <c r="E77" t="n">
+        <v>37229.5</v>
+      </c>
+      <c r="F77" t="n">
+        <v>39396.2</v>
+      </c>
+      <c r="G77" t="n">
+        <v>9277</v>
+      </c>
+      <c r="H77" t="n">
+        <v>10600</v>
+      </c>
+      <c r="I77" t="n">
+        <v>29042</v>
+      </c>
+      <c r="J77" t="n">
+        <v>35814</v>
+      </c>
+      <c r="K77" t="n">
+        <v>38587</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1701.5</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1633.7</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1701</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1727.9</v>
+      </c>
+      <c r="G78" t="n">
+        <v>348</v>
+      </c>
+      <c r="H78" t="n">
+        <v>472</v>
+      </c>
+      <c r="I78" t="n">
+        <v>703</v>
+      </c>
+      <c r="J78" t="n">
+        <v>885</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>16878</v>
+      </c>
+      <c r="D79" t="n">
+        <v>18548</v>
+      </c>
+      <c r="E79" t="n">
+        <v>19368</v>
+      </c>
+      <c r="F79" t="n">
+        <v>19634.9</v>
+      </c>
+      <c r="G79" t="n">
+        <v>8337.627</v>
+      </c>
+      <c r="H79" t="n">
+        <v>14602.112</v>
+      </c>
+      <c r="I79" t="n">
+        <v>21329.168</v>
+      </c>
+      <c r="J79" t="n">
+        <v>22821.343</v>
+      </c>
+      <c r="K79" t="n">
+        <v>23165.256</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>18201</v>
+      </c>
+      <c r="D80" t="n">
+        <v>20743</v>
+      </c>
+      <c r="E80" t="n">
+        <v>21944.7</v>
+      </c>
+      <c r="F80" t="n">
+        <v>25389.5</v>
+      </c>
+      <c r="G80" t="n">
+        <v>15945.909</v>
+      </c>
+      <c r="H80" t="n">
+        <v>17258.28</v>
+      </c>
+      <c r="I80" t="n">
+        <v>16996.382</v>
+      </c>
+      <c r="J80" t="n">
+        <v>19128.085</v>
+      </c>
+      <c r="K80" t="n">
+        <v>21873.498</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - air - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>46940.691</v>
+      </c>
+      <c r="D81" t="n">
+        <v>48734.483</v>
+      </c>
+      <c r="E81" t="n">
+        <v>50695.476</v>
+      </c>
+      <c r="F81" t="n">
+        <v>50253.1</v>
+      </c>
+      <c r="G81" t="n">
+        <v>10932.649</v>
+      </c>
+      <c r="H81" t="n">
+        <v>13735.582</v>
+      </c>
+      <c r="I81" t="n">
+        <v>31938.417</v>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - by land - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>28913.34</v>
+      </c>
+      <c r="D82" t="n">
+        <v>27920.526</v>
+      </c>
+      <c r="E82" t="n">
+        <v>28489.235</v>
+      </c>
+      <c r="F82" t="n">
+        <v>28651.9</v>
+      </c>
+      <c r="G82" t="n">
+        <v>8221.689</v>
+      </c>
+      <c r="H82" t="n">
+        <v>8290.293</v>
+      </c>
+      <c r="I82" t="n">
+        <v>18383.956</v>
+      </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>inbound - trips - transport - water - overnight visitors (tourists)</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
         <v>553.457</v>
       </c>
-      <c r="D59" t="n">
+      <c r="D83" t="n">
         <v>531.737</v>
       </c>
-      <c r="E59" t="n">
+      <c r="E83" t="n">
         <v>561.207</v>
       </c>
-      <c r="F59" t="n">
+      <c r="F83" t="n">
         <v>536.7</v>
       </c>
-      <c r="G59" t="n">
+      <c r="G83" t="n">
         <v>57.676</v>
       </c>
-      <c r="H59" t="n">
+      <c r="H83" t="n">
         <v>74.578</v>
       </c>
-      <c r="I59" t="n">
+      <c r="I83" t="n">
         <v>547.312</v>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>UN_Tourism_inbound_expenditure_12_2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D89" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G89" t="n">
+        <v>2020</v>
+      </c>
+      <c r="H89" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I89" t="n">
+        <v>2022</v>
+      </c>
+      <c r="J89" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K89" t="n">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>inbound - expenditure - balance of payments - total - visitors</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="n">
+        <v>13899.963252617</v>
+      </c>
+      <c r="H90" t="n">
+        <v>15360.7697581997</v>
+      </c>
+      <c r="I90" t="n">
+        <v>31816.9121593968</v>
+      </c>
+      <c r="J90" t="n">
+        <v>45409.9218533883</v>
+      </c>
+      <c r="K90" t="n">
+        <v>49886.0324452887</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>inbound - expenditure - balance of payments - total - visitors</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="n">
+        <v>18380.4147013811</v>
+      </c>
+      <c r="H91" t="n">
+        <v>34176.1559870135</v>
+      </c>
+      <c r="I91" t="n">
+        <v>72083.3294863503</v>
+      </c>
+      <c r="J91" t="n">
+        <v>92144.2801105462</v>
+      </c>
+      <c r="K91" t="n">
+        <v>106656.535197297</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>inbound - expenditure - balance of payments - total - visitors</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>42423</v>
+      </c>
+      <c r="D92" t="n">
+        <v>46719</v>
+      </c>
+      <c r="E92" t="n">
+        <v>51602</v>
+      </c>
+      <c r="F92" t="n">
+        <v>51910</v>
+      </c>
+      <c r="G92" t="n">
+        <v>20316.7578071358</v>
+      </c>
+      <c r="H92" t="n">
+        <v>25354.9279185429</v>
+      </c>
+      <c r="I92" t="n">
+        <v>47100.4319500271</v>
+      </c>
+      <c r="J92" t="n">
+        <v>57919.6252057293</v>
+      </c>
+      <c r="K92" t="n">
+        <v>61433.937023306</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>inbound - expenditure - balance of payments - total - visitors</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>23270</v>
+      </c>
+      <c r="D93" t="n">
+        <v>24619</v>
+      </c>
+      <c r="E93" t="n">
+        <v>26044</v>
+      </c>
+      <c r="F93" t="n">
+        <v>27126</v>
+      </c>
+      <c r="G93" t="n">
+        <v>12142.599224</v>
+      </c>
+      <c r="H93" t="n">
+        <v>22138.069892</v>
+      </c>
+      <c r="I93" t="n">
+        <v>31257.108743</v>
+      </c>
+      <c r="J93" t="n">
+        <v>33495.50487</v>
+      </c>
+      <c r="K93" t="n">
+        <v>36239.253442</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>inbound - expenditure - balance of payments - total - visitors</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>228549</v>
+      </c>
+      <c r="D94" t="n">
+        <v>233758</v>
+      </c>
+      <c r="E94" t="n">
+        <v>241984</v>
+      </c>
+      <c r="F94" t="n">
+        <v>239065</v>
+      </c>
+      <c r="G94" t="n">
+        <v>84297</v>
+      </c>
+      <c r="H94" t="n">
+        <v>84506</v>
+      </c>
+      <c r="I94" t="n">
+        <v>172284</v>
+      </c>
+      <c r="J94" t="n">
+        <v>226167</v>
+      </c>
+      <c r="K94" t="n">
+        <v>251649</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
funcionando como deberia todo
</commit_message>
<xml_diff>
--- a/outputs/world/views_single_sheet.xlsx
+++ b/outputs/world/views_single_sheet.xlsx
@@ -1474,71 +1474,71 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="C59" t="n">
-        <v>2017</v>
+        <v>2022</v>
       </c>
       <c r="D59" t="n">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="E59" t="n">
-        <v>2019</v>
+        <v>2024</v>
       </c>
       <c r="F59" t="n">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="G59" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="H59" t="n">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="I59" t="n">
-        <v>2023</v>
+        <v>2028</v>
       </c>
       <c r="J59" t="n">
-        <v>2024</v>
+        <v>2029</v>
       </c>
       <c r="K59" t="n">
-        <v>2025</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.3049974583544135</v>
+        <v>2.1</v>
       </c>
       <c r="C60" t="n">
-        <v>1.162278697649755</v>
+        <v>5.9</v>
       </c>
       <c r="D60" t="n">
-        <v>2.09910812542079</v>
+        <v>5.7</v>
       </c>
       <c r="E60" t="n">
-        <v>1.298241662778914</v>
+        <v>2.3</v>
       </c>
       <c r="F60" t="n">
-        <v>0.5240757210011437</v>
+        <v>1.1</v>
       </c>
       <c r="G60" t="n">
-        <v>2.066416000505547</v>
+        <v>1.5</v>
       </c>
       <c r="H60" t="n">
-        <v>5.905798223075291</v>
+        <v>1.9</v>
       </c>
       <c r="I60" t="n">
-        <v>5.664155272830939</v>
+        <v>1.9</v>
       </c>
       <c r="J60" t="n">
-        <v>2.317523548694967</v>
+        <v>1.9</v>
       </c>
       <c r="K60" t="n">
-        <v>0.9273716583866166</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="64">

</xml_diff>